<commit_message>
Update Philly BYOB Restaurant_with_websites_20251104_142325.xlsx
</commit_message>
<xml_diff>
--- a/philly_yelp_crawler/data/Philly BYOB Restaurant_with_websites_20251104_142325.xlsx
+++ b/philly_yelp_crawler/data/Philly BYOB Restaurant_with_websites_20251104_142325.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\slow3\OneDrive\桌面\GitHubProjects\BYOB\philly_yelp_crawler\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D20FFEA6-0B17-4479-9ED5-1FAA1915450C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F02DF8B8-3939-477D-A506-4E65CCA5E43C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="241">
   <si>
     <t>Name</t>
   </si>
@@ -734,13 +734,22 @@
   </si>
   <si>
     <t>4728 Baltimore Ave, Philadelphia, PA 19143, United States</t>
+  </si>
+  <si>
+    <t>Porcini</t>
+  </si>
+  <si>
+    <t>2048 Sansom St, Philadelphia, PA 19103</t>
+  </si>
+  <si>
+    <t>(215) 751-1175</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -759,6 +768,14 @@
       <sz val="9"/>
       <name val="新細明體"/>
       <family val="3"/>
+      <charset val="136"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="新細明體"/>
+      <family val="2"/>
       <charset val="136"/>
       <scheme val="minor"/>
     </font>
@@ -798,10 +815,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1105,7 +1125,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="4" max="4" width="27.125" customWidth="1"/>
@@ -2217,8 +2237,23 @@
         <v>15</v>
       </c>
     </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A44" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="H44" t="s">
+        <v>95</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>